<commit_message>
Add cheque and cash deposit slip mapping sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UNYgRRspK6mAkfUf7oZq44
</commit_message>
<xml_diff>
--- a/PA_communication_mapping_tables_20261021_1.xlsx
+++ b/PA_communication_mapping_tables_20261021_1.xlsx
@@ -15,12 +15,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endo Schedule" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tax Invoice" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Receipt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welcome Letter" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premium Details&gt;&gt;" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PC" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GCV" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCV" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2W" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deposit Slip-Cheque" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deposit Slip-Cash" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welcome Letter" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premium Details&gt;&gt;" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PC" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GCV" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCV" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2W" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule-PCAR'!$A$1:$G$1</definedName>
@@ -2866,6 +2868,1751 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>Sr No</t>
+        </is>
+      </c>
+      <c r="B1" s="77" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="77" t="inlineStr">
+        <is>
+          <t>Document Field (Cheque Deposit Slip)</t>
+        </is>
+      </c>
+      <c r="D1" s="77" t="inlineStr">
+        <is>
+          <t>PolicyDD / BCP Field</t>
+        </is>
+      </c>
+      <c r="E1" s="77" t="inlineStr">
+        <is>
+          <t>Associated API</t>
+        </is>
+      </c>
+      <c r="F1" s="77" t="inlineStr">
+        <is>
+          <t>Comments / Customer Clarification</t>
+        </is>
+      </c>
+      <c r="G1" s="77" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Name of Account Holder</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>Fixed/configurable: "Protec Insurance".</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Account Type</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>Configurable, e.g. Current Account.</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Account Number</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>Statement.AccountNo</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Statement carries AccountNo; full account number from bank master.</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Bank Name</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>Configurable per deposit account.</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>Branch Name</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>Configurable per deposit account.</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>IFSC Code</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="n"/>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>Configurable per deposit account.</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Branch Code</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Statement.Office / Collection.BranchCode</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Mapping to Protec Branch code. Office on Statement (e.g. 500100).</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Pickup Address</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Branch address (India Branch module)</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Branch master / India Branch module</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>Combine &lt;address Line 1&gt;, &lt;address Line 2&gt;, &lt;City&gt;, &lt;District&gt;, &lt;State&gt;, &lt;PIN Code&gt;.</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Slip #</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>Statement.StatementNo</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+GET /platform/bcp-core/... statement query (confirm endpoint)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Statement number is the deposit slip number.</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Date of Deposit</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>Statement.Date</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Statement date.</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Total Number of Instruments</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>Count of Statement lines (Cheq/DD)</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>Count of instrument rows in the slip.</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Type</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Collection.PaymentMethod / Statement.InstrumentType</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)
+CodeTable: BcpPaymentMethod</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Local Cheque / Outstation Cheque / Demand Draft. Local vs Outstation needs a flag; confirm source.</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Date</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>Collection.InstrumentDate</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Template shows a date; same as Cheque Date? Confirm with Protec.</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Bank Name (drawee)</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Statement.BankName / Collection.BankName</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Customer cheque bank.</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Branch Name (drawee)</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>Statement.BranchName</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Customer cheque bank branch.</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>IFSC Code (drawee)</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Statement.IFSCCode</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Customer cheque IFSC.</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Cheque No</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Statement.ChequeNo / Collection.InstrumentNo</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Cheque / DD number.</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Cheque Date</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Statement.ChequeDate / Collection.InstrumentDate</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Cheque / DD date.</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Instrument Table</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>Statement.Amount / Collection.Amount</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Per instrument.</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>Totals</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Total Amount</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Sum of Amount</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Sum of instrument amounts (not shown in sample; add if needed).</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Totals</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Amount in Words</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>Derived from total</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>Convert to words in template: Indian Rupees ... and Paisa ... ONLY.</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>Signature and Stamp - Protec General Insurance</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank; fixed wording "Protec General Insurance".</t>
+        </is>
+      </c>
+      <c r="G23" s="23" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>Date (Protec)</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
+      <c r="F24" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank.</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Signature and Stamp - Bank Collection Agent</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank; fixed wording.</t>
+        </is>
+      </c>
+      <c r="G25" s="23" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>Date (Bank)</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank.</t>
+        </is>
+      </c>
+      <c r="G26" s="23" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="78" t="inlineStr">
+        <is>
+          <t>Associated API reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="79" t="inlineStr">
+        <is>
+          <t>API purpose</t>
+        </is>
+      </c>
+      <c r="C30" s="79" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D30" s="79" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="80" t="inlineStr">
+        <is>
+          <t>Statement (deposit slip header + lines)</t>
+        </is>
+      </c>
+      <c r="C31" s="80" t="inlineStr">
+        <is>
+          <t>BCP Statement page (bcp-core); Statement fields: StatementNo, Office, AccountNo, Date, Cash/Cheque, InstrumentType, Bank/Branch/IFSC, Cheque No/Date, Amount, denominations</t>
+        </is>
+      </c>
+      <c r="D31" s="80" t="inlineStr">
+        <is>
+          <t>Exact statement endpoint not in the BCP query skill; confirm with BCP team. URL via client.py get-url --page statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="80" t="inlineStr">
+        <is>
+          <t>Collection search</t>
+        </is>
+      </c>
+      <c r="C32" s="80" t="inlineStr">
+        <is>
+          <t>POST /platform/bcp-core/query/v1/queryEsData</t>
+        </is>
+      </c>
+      <c r="D32" s="80" t="inlineStr">
+        <is>
+          <t>Module=Collection; filter by ReceiptNo / CollectionNo / PolicyNo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="80" t="inlineStr">
+        <is>
+          <t>Collection by ID</t>
+        </is>
+      </c>
+      <c r="C33" s="80" t="inlineStr">
+        <is>
+          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
+      <c r="D33" s="80" t="inlineStr">
+        <is>
+          <t>ID must be signed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="80" t="inlineStr">
+        <is>
+          <t>Offset / Statement offset</t>
+        </is>
+      </c>
+      <c r="C34" s="80" t="inlineStr">
+        <is>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Offset)</t>
+        </is>
+      </c>
+      <c r="D34" s="80" t="inlineStr">
+        <is>
+          <t>Offset record has StatementNo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="80" t="inlineStr">
+        <is>
+          <t>Code tables</t>
+        </is>
+      </c>
+      <c r="C35" s="80" t="inlineStr">
+        <is>
+          <t>BcpPaymentMethod, BcpCollectionType</t>
+        </is>
+      </c>
+      <c r="D35" s="80" t="inlineStr">
+        <is>
+          <t>Instrument type descriptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="80" t="inlineStr">
+        <is>
+          <t>Document generation</t>
+        </is>
+      </c>
+      <c r="C36" s="80" t="inlineStr">
+        <is>
+          <t>InsureMO Output Service: template upload + print task (PDF)</t>
+        </is>
+      </c>
+      <c r="D36" s="80" t="inlineStr">
+        <is>
+          <t>Handlebars template from the Excel slip.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>Sr No</t>
+        </is>
+      </c>
+      <c r="B1" s="77" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="77" t="inlineStr">
+        <is>
+          <t>Document Field (Cash Deposit Slip)</t>
+        </is>
+      </c>
+      <c r="D1" s="77" t="inlineStr">
+        <is>
+          <t>PolicyDD / BCP Field</t>
+        </is>
+      </c>
+      <c r="E1" s="77" t="inlineStr">
+        <is>
+          <t>Associated API</t>
+        </is>
+      </c>
+      <c r="F1" s="77" t="inlineStr">
+        <is>
+          <t>Comments / Customer Clarification</t>
+        </is>
+      </c>
+      <c r="G1" s="77" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Name of Account Holder</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>Fixed/configurable: "Protec Insurance".</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Account Type</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>Configurable, e.g. Current Account.</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Account Number</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>Statement.AccountNo</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Statement carries AccountNo; full account number from bank master.</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Bank Name</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>Configurable per deposit account.</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>Branch Name</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>Configurable per deposit account.</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Bank Account (Header)</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>IFSC Code</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="n"/>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Company bank account master (Protec) - configurable</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>Configurable per deposit account.</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>Pending Protec provide before go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Branch Code</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Statement.Office / Collection.BranchCode</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+POST /platform/bcp-core/query/v1/queryEsData (Module=Collection)</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Mapping to Protec Branch code. Office on Statement (e.g. 500100).</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Pickup Address</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Branch address (India Branch module)</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Branch master / India Branch module</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>Combine &lt;address Line 1&gt;, &lt;address Line 2&gt;, &lt;City&gt;, &lt;District&gt;, &lt;State&gt;, &lt;PIN Code&gt;.</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Slip #</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>Statement.StatementNo</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"
+GET /platform/bcp-core/... statement query (confirm endpoint)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Statement number is the deposit slip number.</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Deposit Info (Header)</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Date of Deposit</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>Statement.Date</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Statement date.</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Denomination Table</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>Notes / Coins (fixed)</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="n"/>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>Fixed lines: Notes 500,100,50,20,10; Coins 20,10,5,2,1.</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Denomination Table</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Denomination</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Statement columns 500/100/50/20/10/1</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Statement carries denomination columns (Notes 500..10, Coins 1). Coins 20/10/5/2 not in Statement; confirm.</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Denomination Table</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Pieces</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>Statement.&lt;denomination&gt; count</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>BCP Statement (bcp-core) - page "statement"</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Piece count per denomination.</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Denomination Table</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Denomination x Pieces</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="n"/>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Calculated in template.</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Denomination Table</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="n"/>
+      <c r="E16" s="23" t="n"/>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank / free text.</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>Totals</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Sum of Amount</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Sum of denomination amounts; must equal Collection.Amount for the statement.</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Totals</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Amount in Words</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Derived from total</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="n"/>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Convert to words in template: Indian Rupees ... and Paisa ... ONLY.</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Signature and Stamp - Protec General Insurance</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="n"/>
+      <c r="E19" s="23" t="n"/>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank; fixed wording.</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>Date (Protec)</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank.</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Signature and Stamp - Bank Collection Agent</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank; fixed wording.</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Date (Bank)</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>Keep blank.</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="78" t="inlineStr">
+        <is>
+          <t>Associated API reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="79" t="inlineStr">
+        <is>
+          <t>API purpose</t>
+        </is>
+      </c>
+      <c r="C26" s="79" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D26" s="79" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="80" t="inlineStr">
+        <is>
+          <t>Statement (deposit slip header + lines)</t>
+        </is>
+      </c>
+      <c r="C27" s="80" t="inlineStr">
+        <is>
+          <t>BCP Statement page (bcp-core); Statement fields: StatementNo, Office, AccountNo, Date, Cash/Cheque, InstrumentType, Bank/Branch/IFSC, Cheque No/Date, Amount, denominations</t>
+        </is>
+      </c>
+      <c r="D27" s="80" t="inlineStr">
+        <is>
+          <t>Exact statement endpoint not in the BCP query skill; confirm with BCP team. URL via client.py get-url --page statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="80" t="inlineStr">
+        <is>
+          <t>Collection search</t>
+        </is>
+      </c>
+      <c r="C28" s="80" t="inlineStr">
+        <is>
+          <t>POST /platform/bcp-core/query/v1/queryEsData</t>
+        </is>
+      </c>
+      <c r="D28" s="80" t="inlineStr">
+        <is>
+          <t>Module=Collection; filter by ReceiptNo / CollectionNo / PolicyNo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="80" t="inlineStr">
+        <is>
+          <t>Collection by ID</t>
+        </is>
+      </c>
+      <c r="C29" s="80" t="inlineStr">
+        <is>
+          <t>GET /platform/bcp-core/collection/v1/getCollection</t>
+        </is>
+      </c>
+      <c r="D29" s="80" t="inlineStr">
+        <is>
+          <t>ID must be signed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="80" t="inlineStr">
+        <is>
+          <t>Offset / Statement offset</t>
+        </is>
+      </c>
+      <c r="C30" s="80" t="inlineStr">
+        <is>
+          <t>POST /platform/bcp-core/query/v1/queryEsData (Module=Offset)</t>
+        </is>
+      </c>
+      <c r="D30" s="80" t="inlineStr">
+        <is>
+          <t>Offset record has StatementNo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="80" t="inlineStr">
+        <is>
+          <t>Code tables</t>
+        </is>
+      </c>
+      <c r="C31" s="80" t="inlineStr">
+        <is>
+          <t>BcpPaymentMethod, BcpCollectionType</t>
+        </is>
+      </c>
+      <c r="D31" s="80" t="inlineStr">
+        <is>
+          <t>Instrument type descriptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="80" t="inlineStr">
+        <is>
+          <t>Document generation</t>
+        </is>
+      </c>
+      <c r="C32" s="80" t="inlineStr">
+        <is>
+          <t>InsureMO Output Service: template upload + print task (PDF)</t>
+        </is>
+      </c>
+      <c r="D32" s="80" t="inlineStr">
+        <is>
+          <t>Handlebars template from the Excel slip.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2885,7 +4632,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2898,7 +4645,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -3657,7 +5404,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -4634,7 +6381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -5408,7 +7155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>

</xml_diff>